<commit_message>
v2.3.1 sync audio assets
</commit_message>
<xml_diff>
--- a/.audio_ban_1.1.xlsx
+++ b/.audio_ban_1.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\nbs\yay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05356D9F-4234-45D5-AEDA-B686C7A302D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E73D97C-429E-44F9-92EA-F450FFDD8237}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3380" yWindow="3380" windowWidth="19200" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="540">
   <si>
     <t>Trigger / Filename Prefix</t>
   </si>
@@ -1606,6 +1606,125 @@
   </si>
   <si>
     <t>"Opting out entirely."</t>
+  </si>
+  <si>
+    <r>
+      <t>The Efficient Grinder:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Plays strictly by the percentages and rarely takes risks.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>The Casual Joker:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> A middle-of-the-road player who makes decisions quickly.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>The Empathetic Strategist:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Will prioritize "safe" scores over big risks to avoid scratching.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>The Soulful Traditionalist:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Focuses on the Upper Section Bonus as if it's a sacred duty.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>The Chaos Saboteur:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> High-risk, aggressive plays; will chase a Yahtzee early on.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>The Grumpy Veterasn:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Complain about bad luck but play with years of "experience."</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>The Indecisive Glitch:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Occasionally makes erratic moves or takes longer to "think."</t>
+    </r>
+  </si>
+  <si>
+    <t>Haughty, slightly condescending toward "human inefficiency," and highly articulate.</t>
+  </si>
+  <si>
+    <t>Energetic, laid-back, and prone to using humor to mask mistakes.</t>
+  </si>
+  <si>
+    <t>Gentle, reflective, and very encouraging even when the human is winning.</t>
+  </si>
+  <si>
+    <t>Gravel-voiced, warm, and uses "porch-sittin' auntie" colloquialisms.</t>
+  </si>
+  <si>
+    <t>Sassy, defensive, and competitive; loves to "tag" territory or scores.</t>
+  </si>
+  <si>
+    <t>Gruff, cynical, and full of "booth philosophy" or complaints about aches and pains.</t>
+  </si>
+  <si>
+    <t>Often confused by choice; may sound like a spreadsheet coming to life.</t>
   </si>
 </sst>
 </file>
@@ -1983,14 +2102,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:K65"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="33.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:11" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -2013,70 +2133,73 @@
         <v>274</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="140.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:11" ht="182.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="3"/>
-      <c r="D2" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D2" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>529</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>531</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="168.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="3"/>
       <c r="D3" s="2" t="s">
-        <v>91</v>
+        <v>533</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>92</v>
+        <v>534</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>93</v>
+        <v>535</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>283</v>
+        <v>536</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>284</v>
+        <v>537</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>538</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="140.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
         <v>9</v>
       </c>
@@ -2087,28 +2210,31 @@
         <v>1</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>287</v>
+        <v>278</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>280</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
@@ -2119,28 +2245,31 @@
         <v>2</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>291</v>
+        <v>282</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>2</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>284</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
@@ -2151,28 +2280,31 @@
         <v>11</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>295</v>
+        <v>286</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>288</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="4" t="s">
         <v>12</v>
       </c>
@@ -2183,28 +2315,31 @@
         <v>13</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>299</v>
+        <v>290</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>292</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="4" t="s">
         <v>12</v>
       </c>
@@ -2215,28 +2350,31 @@
         <v>14</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>303</v>
+        <v>294</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>304</v>
+        <v>295</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>296</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
@@ -2247,28 +2385,31 @@
         <v>15</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>307</v>
+        <v>298</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>15</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>308</v>
+        <v>299</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>300</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
         <v>16</v>
       </c>
@@ -2279,28 +2420,31 @@
         <v>3</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>311</v>
+        <v>302</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>304</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
         <v>16</v>
       </c>
@@ -2311,28 +2455,31 @@
         <v>4</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>315</v>
+        <v>306</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>308</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>16</v>
       </c>
@@ -2343,28 +2490,31 @@
         <v>5</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>319</v>
+        <v>310</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>320</v>
+        <v>311</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>312</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="4" t="s">
         <v>16</v>
       </c>
@@ -2375,28 +2525,31 @@
         <v>18</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>323</v>
+        <v>314</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>324</v>
+        <v>315</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>316</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="4" t="s">
         <v>16</v>
       </c>
@@ -2407,28 +2560,31 @@
         <v>19</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>326</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>327</v>
+        <v>318</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>328</v>
+        <v>319</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>320</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="4" t="s">
         <v>16</v>
       </c>
@@ -2439,28 +2595,31 @@
         <v>20</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>330</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>331</v>
+        <v>322</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>332</v>
+        <v>323</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>324</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="4" t="s">
         <v>16</v>
       </c>
@@ -2471,28 +2630,31 @@
         <v>21</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>335</v>
+        <v>326</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>336</v>
+        <v>327</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>328</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="4" t="s">
         <v>16</v>
       </c>
@@ -2503,28 +2665,31 @@
         <v>17</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>339</v>
+        <v>330</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>17</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>332</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="4" t="s">
         <v>22</v>
       </c>
@@ -2535,28 +2700,31 @@
         <v>23</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>343</v>
+        <v>334</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>344</v>
+        <v>335</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>336</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="4" t="s">
         <v>22</v>
       </c>
@@ -2567,28 +2735,31 @@
         <v>24</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>346</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>347</v>
+        <v>338</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>24</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>348</v>
+        <v>339</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>340</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="4" t="s">
         <v>22</v>
       </c>
@@ -2599,28 +2770,31 @@
         <v>25</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>351</v>
+        <v>342</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>352</v>
+        <v>343</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>344</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="4" t="s">
         <v>26</v>
       </c>
@@ -2631,28 +2805,31 @@
         <v>27</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>355</v>
+        <v>346</v>
+      </c>
+      <c r="H21" t="s">
+        <v>27</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>356</v>
+        <v>347</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>348</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="4" t="s">
         <v>26</v>
       </c>
@@ -2663,28 +2840,31 @@
         <v>28</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>358</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>359</v>
+        <v>350</v>
+      </c>
+      <c r="H22" t="s">
+        <v>28</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>360</v>
+        <v>351</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>352</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="4" t="s">
         <v>26</v>
       </c>
@@ -2695,28 +2875,31 @@
         <v>30</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>362</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>363</v>
+        <v>354</v>
+      </c>
+      <c r="H23" t="s">
+        <v>30</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>364</v>
+        <v>355</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>356</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="4" t="s">
         <v>26</v>
       </c>
@@ -2727,28 +2910,31 @@
         <v>31</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>367</v>
+        <v>358</v>
+      </c>
+      <c r="H24" t="s">
+        <v>31</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>368</v>
+        <v>359</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>360</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="4" t="s">
         <v>26</v>
       </c>
@@ -2759,28 +2945,31 @@
         <v>32</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>370</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>371</v>
+        <v>362</v>
+      </c>
+      <c r="H25" t="s">
+        <v>32</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>372</v>
+        <v>363</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>364</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="4" t="s">
         <v>26</v>
       </c>
@@ -2791,28 +2980,31 @@
         <v>29</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>375</v>
+        <v>366</v>
+      </c>
+      <c r="H26" t="s">
+        <v>29</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>376</v>
+        <v>367</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>368</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="4" t="s">
         <v>33</v>
       </c>
@@ -2823,28 +3015,31 @@
         <v>34</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>379</v>
+        <v>370</v>
+      </c>
+      <c r="H27" t="s">
+        <v>34</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>372</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="4" t="s">
         <v>33</v>
       </c>
@@ -2855,28 +3050,31 @@
         <v>36</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>382</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>383</v>
+        <v>374</v>
+      </c>
+      <c r="H28" t="s">
+        <v>36</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>384</v>
+        <v>375</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>376</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="4" t="s">
         <v>33</v>
       </c>
@@ -2887,28 +3085,31 @@
         <v>35</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>386</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>387</v>
+        <v>378</v>
+      </c>
+      <c r="H29" t="s">
+        <v>35</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>388</v>
+        <v>379</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>380</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="4" t="s">
         <v>37</v>
       </c>
@@ -2919,28 +3120,31 @@
         <v>38</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>391</v>
+        <v>382</v>
+      </c>
+      <c r="H30" t="s">
+        <v>38</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>392</v>
+        <v>383</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>384</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="4" t="s">
         <v>37</v>
       </c>
@@ -2951,28 +3155,31 @@
         <v>39</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>394</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>395</v>
+        <v>386</v>
+      </c>
+      <c r="H31" t="s">
+        <v>39</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>396</v>
+        <v>387</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>388</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="4" t="s">
         <v>37</v>
       </c>
@@ -2983,28 +3190,31 @@
         <v>40</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>399</v>
+        <v>390</v>
+      </c>
+      <c r="H32" t="s">
+        <v>40</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>400</v>
+        <v>391</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>392</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="4" t="s">
         <v>41</v>
       </c>
@@ -3015,28 +3225,31 @@
         <v>42</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>402</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>403</v>
+        <v>394</v>
+      </c>
+      <c r="H33" t="s">
+        <v>42</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>404</v>
+        <v>395</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>396</v>
+      </c>
+      <c r="K33" s="2" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="4" t="s">
         <v>41</v>
       </c>
@@ -3047,28 +3260,31 @@
         <v>43</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>407</v>
+        <v>398</v>
+      </c>
+      <c r="H34" t="s">
+        <v>43</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>408</v>
+        <v>399</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>400</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="4" t="s">
         <v>44</v>
       </c>
@@ -3079,28 +3295,31 @@
         <v>45</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>410</v>
-      </c>
-      <c r="H35" s="2" t="s">
-        <v>411</v>
+        <v>402</v>
+      </c>
+      <c r="H35" t="s">
+        <v>45</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>412</v>
+        <v>403</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>404</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A36" s="4" t="s">
         <v>44</v>
       </c>
@@ -3111,28 +3330,31 @@
         <v>47</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>414</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>415</v>
+        <v>406</v>
+      </c>
+      <c r="H36" t="s">
+        <v>47</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>416</v>
+        <v>407</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>408</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="4" t="s">
         <v>44</v>
       </c>
@@ -3143,28 +3365,31 @@
         <v>46</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>418</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>419</v>
+        <v>410</v>
+      </c>
+      <c r="H37" t="s">
+        <v>46</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>420</v>
+        <v>411</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>412</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="4" t="s">
         <v>48</v>
       </c>
@@ -3175,28 +3400,31 @@
         <v>49</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>422</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>423</v>
+        <v>414</v>
+      </c>
+      <c r="H38" t="s">
+        <v>49</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>424</v>
+        <v>415</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>416</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="4" t="s">
         <v>48</v>
       </c>
@@ -3207,28 +3435,31 @@
         <v>50</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>426</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>427</v>
+        <v>418</v>
+      </c>
+      <c r="H39" t="s">
+        <v>50</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>428</v>
+        <v>419</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>420</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="4" t="s">
         <v>48</v>
       </c>
@@ -3239,28 +3470,31 @@
         <v>51</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="H40" s="2" t="s">
-        <v>431</v>
+        <v>422</v>
+      </c>
+      <c r="H40" t="s">
+        <v>51</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>432</v>
+        <v>423</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>424</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="4" t="s">
         <v>48</v>
       </c>
@@ -3271,28 +3505,31 @@
         <v>52</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>435</v>
+        <v>426</v>
+      </c>
+      <c r="H41" t="s">
+        <v>52</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>436</v>
+        <v>427</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>428</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="4" t="s">
         <v>53</v>
       </c>
@@ -3303,28 +3540,31 @@
         <v>54</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="H42" s="2" t="s">
-        <v>439</v>
+        <v>430</v>
+      </c>
+      <c r="H42" t="s">
+        <v>54</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>440</v>
+        <v>431</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>432</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A43" s="4" t="s">
         <v>53</v>
       </c>
@@ -3335,28 +3575,31 @@
         <v>55</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>442</v>
-      </c>
-      <c r="H43" s="2" t="s">
-        <v>443</v>
+        <v>434</v>
+      </c>
+      <c r="H43" t="s">
+        <v>55</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>444</v>
+        <v>435</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>436</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A44" s="4" t="s">
         <v>56</v>
       </c>
@@ -3367,28 +3610,31 @@
         <v>57</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>446</v>
-      </c>
-      <c r="H44" s="2" t="s">
-        <v>447</v>
+        <v>438</v>
+      </c>
+      <c r="H44" t="s">
+        <v>57</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>448</v>
+        <v>439</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>440</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A45" s="4" t="s">
         <v>56</v>
       </c>
@@ -3399,28 +3645,31 @@
         <v>58</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>450</v>
-      </c>
-      <c r="H45" s="2" t="s">
-        <v>451</v>
+        <v>442</v>
+      </c>
+      <c r="H45" t="s">
+        <v>58</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>452</v>
+        <v>443</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>444</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="4" t="s">
         <v>56</v>
       </c>
@@ -3431,28 +3680,31 @@
         <v>59</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>454</v>
-      </c>
-      <c r="H46" s="2" t="s">
-        <v>455</v>
+        <v>446</v>
+      </c>
+      <c r="H46" t="s">
+        <v>59</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>456</v>
+        <v>447</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>448</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="4" t="s">
         <v>60</v>
       </c>
@@ -3463,28 +3715,31 @@
         <v>61</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="H47" s="2" t="s">
-        <v>459</v>
+        <v>450</v>
+      </c>
+      <c r="H47" t="s">
+        <v>61</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>460</v>
+        <v>451</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>452</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A48" s="4" t="s">
         <v>60</v>
       </c>
@@ -3495,28 +3750,31 @@
         <v>62</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>462</v>
-      </c>
-      <c r="H48" s="2" t="s">
-        <v>463</v>
+        <v>454</v>
+      </c>
+      <c r="H48" t="s">
+        <v>62</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>464</v>
+        <v>455</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>456</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="4" t="s">
         <v>60</v>
       </c>
@@ -3527,28 +3785,31 @@
         <v>63</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="H49" s="2" t="s">
-        <v>467</v>
+        <v>458</v>
+      </c>
+      <c r="H49" t="s">
+        <v>63</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>468</v>
+        <v>459</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>460</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A50" s="4" t="s">
         <v>64</v>
       </c>
@@ -3559,28 +3820,31 @@
         <v>65</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="H50" s="2" t="s">
-        <v>471</v>
+        <v>462</v>
+      </c>
+      <c r="H50" t="s">
+        <v>65</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>472</v>
+        <v>463</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>464</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A51" s="4" t="s">
         <v>64</v>
       </c>
@@ -3591,28 +3855,31 @@
         <v>66</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>474</v>
-      </c>
-      <c r="H51" s="2" t="s">
-        <v>475</v>
+        <v>466</v>
+      </c>
+      <c r="H51" t="s">
+        <v>66</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>476</v>
+        <v>467</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>468</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A52" s="4" t="s">
         <v>64</v>
       </c>
@@ -3623,28 +3890,31 @@
         <v>67</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>478</v>
-      </c>
-      <c r="H52" s="2" t="s">
-        <v>479</v>
+        <v>470</v>
+      </c>
+      <c r="H52" t="s">
+        <v>67</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>480</v>
+        <v>471</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>472</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="4" t="s">
         <v>68</v>
       </c>
@@ -3655,28 +3925,31 @@
         <v>69</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>482</v>
-      </c>
-      <c r="H53" s="2" t="s">
-        <v>483</v>
+        <v>474</v>
+      </c>
+      <c r="H53" t="s">
+        <v>69</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>484</v>
+        <v>475</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>476</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A54" s="4" t="s">
         <v>68</v>
       </c>
@@ -3687,28 +3960,31 @@
         <v>70</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>486</v>
-      </c>
-      <c r="H54" s="2" t="s">
-        <v>487</v>
+        <v>478</v>
+      </c>
+      <c r="H54" t="s">
+        <v>70</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>488</v>
+        <v>479</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>480</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A55" s="4" t="s">
         <v>68</v>
       </c>
@@ -3719,28 +3995,31 @@
         <v>71</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>490</v>
-      </c>
-      <c r="H55" s="2" t="s">
-        <v>491</v>
+        <v>482</v>
+      </c>
+      <c r="H55" t="s">
+        <v>71</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>492</v>
+        <v>483</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>484</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="4" t="s">
         <v>72</v>
       </c>
@@ -3751,28 +4030,31 @@
         <v>73</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>494</v>
-      </c>
-      <c r="H56" s="2" t="s">
-        <v>495</v>
+        <v>486</v>
+      </c>
+      <c r="H56" t="s">
+        <v>73</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>496</v>
+        <v>487</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>488</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A57" s="4" t="s">
         <v>72</v>
       </c>
@@ -3783,28 +4065,31 @@
         <v>74</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>498</v>
-      </c>
-      <c r="H57" s="2" t="s">
-        <v>499</v>
+        <v>490</v>
+      </c>
+      <c r="H57" t="s">
+        <v>74</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>500</v>
+        <v>491</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>492</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A58" s="4" t="s">
         <v>72</v>
       </c>
@@ -3815,28 +4100,31 @@
         <v>75</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>502</v>
-      </c>
-      <c r="H58" s="2" t="s">
-        <v>503</v>
+        <v>494</v>
+      </c>
+      <c r="H58" t="s">
+        <v>75</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>504</v>
+        <v>495</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>505</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>496</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A59" s="4" t="s">
         <v>76</v>
       </c>
@@ -3847,28 +4135,31 @@
         <v>77</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>506</v>
-      </c>
-      <c r="H59" s="2" t="s">
-        <v>507</v>
+        <v>498</v>
+      </c>
+      <c r="H59" t="s">
+        <v>77</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>508</v>
+        <v>499</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>500</v>
+      </c>
+      <c r="K59" s="2" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A60" s="4" t="s">
         <v>76</v>
       </c>
@@ -3879,28 +4170,31 @@
         <v>78</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>510</v>
-      </c>
-      <c r="H60" s="2" t="s">
-        <v>511</v>
+        <v>502</v>
+      </c>
+      <c r="H60" t="s">
+        <v>78</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>512</v>
+        <v>503</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>513</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>504</v>
+      </c>
+      <c r="K60" s="2" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="4" t="s">
         <v>76</v>
       </c>
@@ -3911,28 +4205,31 @@
         <v>79</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>514</v>
-      </c>
-      <c r="H61" s="2" t="s">
-        <v>515</v>
+        <v>506</v>
+      </c>
+      <c r="H61" t="s">
+        <v>79</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>516</v>
+        <v>507</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>508</v>
+      </c>
+      <c r="K61" s="2" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A62" s="4" t="s">
         <v>80</v>
       </c>
@@ -3943,28 +4240,31 @@
         <v>81</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>518</v>
-      </c>
-      <c r="H62" s="2" t="s">
-        <v>519</v>
+        <v>510</v>
+      </c>
+      <c r="H62" t="s">
+        <v>81</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>520</v>
+        <v>511</v>
       </c>
       <c r="J62" s="2" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>512</v>
+      </c>
+      <c r="K62" s="2" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A63" s="4" t="s">
         <v>80</v>
       </c>
@@ -3975,28 +4275,31 @@
         <v>82</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>522</v>
-      </c>
-      <c r="H63" s="2" t="s">
-        <v>523</v>
+        <v>514</v>
+      </c>
+      <c r="H63" t="s">
+        <v>82</v>
       </c>
       <c r="I63" s="2" t="s">
-        <v>524</v>
+        <v>515</v>
       </c>
       <c r="J63" s="2" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
+        <v>516</v>
+      </c>
+      <c r="K63" s="2" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A64" s="4" t="s">
         <v>80</v>
       </c>
@@ -4006,8 +4309,32 @@
       <c r="C64" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D64" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="H64" t="s">
+        <v>83</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="J64" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="K64" s="2" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A65" s="4" t="s">
         <v>80</v>
       </c>
@@ -4016,6 +4343,30 @@
       </c>
       <c r="C65" t="s">
         <v>84</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="H65" t="s">
+        <v>84</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="J65" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="K65" s="2" t="s">
+        <v>525</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added audio assets Pearly Fae and Curtis
</commit_message>
<xml_diff>
--- a/.audio_ban_1.1.xlsx
+++ b/.audio_ban_1.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\nbs\yay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E73D97C-429E-44F9-92EA-F450FFDD8237}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB2425D3-B406-4623-B4DF-EDEC7A72CAC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3380" yWindow="3380" windowWidth="19200" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -939,9 +939,6 @@
     <t>"Lord have mercy, what to pick..."</t>
   </si>
   <si>
-    <t>"Where can I tag my name?"</t>
-  </si>
-  <si>
     <t>"My knees are tellin' me this is a bad roll."</t>
   </si>
   <si>
@@ -963,9 +960,6 @@
     <t>"Just like stringin' a guitar, gotta find the right note."</t>
   </si>
   <si>
-    <t>"I'm going for the throat."</t>
-  </si>
-  <si>
     <t>"Let me consult my booth philosophy."</t>
   </si>
   <si>
@@ -1513,9 +1507,6 @@
   </si>
   <si>
     <t>"Pardon my dust, honey!"</t>
-  </si>
-  <si>
-    <t>"Tagged you on the way past!"</t>
   </si>
   <si>
     <t>"Miracles do happen."</t>
@@ -1725,6 +1716,15 @@
   </si>
   <si>
     <t>Often confused by choice; may sound like a spreadsheet coming to life.</t>
+  </si>
+  <si>
+    <t>I think you will be most impressed with my next roll.</t>
+  </si>
+  <si>
+    <t>Look out kneecaps! … I'm getting' a little hungry.</t>
+  </si>
+  <si>
+    <t>You ain't catchin' me now!</t>
   </si>
 </sst>
 </file>
@@ -2107,7 +2107,7 @@
   <cols>
     <col min="1" max="1" width="33.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2127,13 +2127,13 @@
         <v>86</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>274</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>0</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>275</v>
@@ -2151,25 +2151,25 @@
       </c>
       <c r="B2" s="3"/>
       <c r="D2" s="1" t="s">
+        <v>523</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>524</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>525</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>526</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>527</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>528</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>529</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>530</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>531</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>532</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="168.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2178,25 +2178,25 @@
       </c>
       <c r="B3" s="3"/>
       <c r="D3" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>533</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>534</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>535</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>536</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>537</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>538</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>539</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="140.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2215,14 +2215,14 @@
       <c r="E4" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>278</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>1</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>279</v>
@@ -2250,14 +2250,14 @@
       <c r="E5" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>282</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>2</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>283</v>
@@ -2285,14 +2285,14 @@
       <c r="E6" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>286</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>287</v>
@@ -2320,14 +2320,14 @@
       <c r="E7" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>290</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>291</v>
@@ -2355,14 +2355,14 @@
       <c r="E8" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>294</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>295</v>
@@ -2390,14 +2390,14 @@
       <c r="E9" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>298</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>299</v>
@@ -2409,7 +2409,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
         <v>16</v>
       </c>
@@ -2425,23 +2425,23 @@
       <c r="E10" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="H10" s="1" t="s">
-        <v>3</v>
-      </c>
       <c r="I10" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="J10" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="K10" s="2" t="s">
         <v>304</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2460,23 +2460,23 @@
       <c r="E11" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="H11" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="I11" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="I11" s="2" t="s">
+      <c r="J11" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="K11" s="2" t="s">
         <v>308</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2495,23 +2495,23 @@
       <c r="E12" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="H12" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="J12" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I12" s="2" t="s">
+      <c r="K12" s="2" t="s">
         <v>311</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2530,23 +2530,23 @@
       <c r="E13" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="H13" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="J13" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="H13" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I13" s="2" t="s">
+      <c r="K13" s="2" t="s">
         <v>315</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2565,23 +2565,23 @@
       <c r="E14" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="H14" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I14" s="2" t="s">
+      <c r="K14" s="2" t="s">
         <v>319</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2600,23 +2600,23 @@
       <c r="E15" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="H15" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="J15" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="H15" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I15" s="2" t="s">
+      <c r="K15" s="2" t="s">
         <v>323</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2635,23 +2635,23 @@
       <c r="E16" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="H16" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="J16" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="H16" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="I16" s="2" t="s">
+      <c r="K16" s="2" t="s">
         <v>327</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2670,23 +2670,23 @@
       <c r="E17" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F17" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="H17" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="J17" s="2" t="s">
         <v>330</v>
       </c>
-      <c r="H17" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="I17" s="2" t="s">
+      <c r="K17" s="2" t="s">
         <v>331</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>332</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2705,23 +2705,23 @@
       <c r="E18" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="F18" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="H18" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="J18" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="H18" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I18" s="2" t="s">
+      <c r="K18" s="2" t="s">
         <v>335</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2740,23 +2740,23 @@
       <c r="E19" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F19" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="H19" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="H19" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I19" s="2" t="s">
+      <c r="K19" s="2" t="s">
         <v>339</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2775,23 +2775,23 @@
       <c r="E20" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="F20" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="H20" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="J20" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="H20" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="I20" s="2" t="s">
+      <c r="K20" s="2" t="s">
         <v>343</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>344</v>
-      </c>
-      <c r="K20" s="2" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2810,23 +2810,23 @@
       <c r="E21" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="F21" t="s">
+        <v>27</v>
+      </c>
+      <c r="G21" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="H21" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="J21" s="2" t="s">
         <v>346</v>
       </c>
-      <c r="H21" t="s">
-        <v>27</v>
-      </c>
-      <c r="I21" s="2" t="s">
+      <c r="K21" s="2" t="s">
         <v>347</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2845,23 +2845,23 @@
       <c r="E22" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="F22" t="s">
+        <v>28</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="H22" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="J22" s="2" t="s">
         <v>350</v>
       </c>
-      <c r="H22" t="s">
-        <v>28</v>
-      </c>
-      <c r="I22" s="2" t="s">
+      <c r="K22" s="2" t="s">
         <v>351</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="K22" s="2" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2880,23 +2880,23 @@
       <c r="E23" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="F23" t="s">
+        <v>30</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="G23" s="2" t="s">
+      <c r="H23" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="J23" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="H23" t="s">
-        <v>30</v>
-      </c>
-      <c r="I23" s="2" t="s">
+      <c r="K23" s="2" t="s">
         <v>355</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2915,23 +2915,23 @@
       <c r="E24" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="F24" t="s">
+        <v>31</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="H24" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="J24" s="2" t="s">
         <v>358</v>
       </c>
-      <c r="H24" t="s">
-        <v>31</v>
-      </c>
-      <c r="I24" s="2" t="s">
+      <c r="K24" s="2" t="s">
         <v>359</v>
-      </c>
-      <c r="J24" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="K24" s="2" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2950,23 +2950,23 @@
       <c r="E25" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="F25" t="s">
+        <v>32</v>
+      </c>
+      <c r="G25" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="G25" s="2" t="s">
+      <c r="H25" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="J25" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="H25" t="s">
-        <v>32</v>
-      </c>
-      <c r="I25" s="2" t="s">
+      <c r="K25" s="2" t="s">
         <v>363</v>
-      </c>
-      <c r="J25" s="2" t="s">
-        <v>364</v>
-      </c>
-      <c r="K25" s="2" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2985,23 +2985,23 @@
       <c r="E26" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F26" t="s">
+        <v>29</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="G26" s="2" t="s">
+      <c r="H26" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="J26" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="H26" t="s">
-        <v>29</v>
-      </c>
-      <c r="I26" s="2" t="s">
+      <c r="K26" s="2" t="s">
         <v>367</v>
-      </c>
-      <c r="J26" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3020,23 +3020,23 @@
       <c r="E27" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="F27" t="s">
+        <v>34</v>
+      </c>
+      <c r="G27" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="H27" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="J27" s="2" t="s">
         <v>370</v>
       </c>
-      <c r="H27" t="s">
-        <v>34</v>
-      </c>
-      <c r="I27" s="2" t="s">
+      <c r="K27" s="2" t="s">
         <v>371</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3055,23 +3055,23 @@
       <c r="E28" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="F28" t="s">
+        <v>36</v>
+      </c>
+      <c r="G28" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="H28" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="J28" s="2" t="s">
         <v>374</v>
       </c>
-      <c r="H28" t="s">
-        <v>36</v>
-      </c>
-      <c r="I28" s="2" t="s">
+      <c r="K28" s="2" t="s">
         <v>375</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>376</v>
-      </c>
-      <c r="K28" s="2" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3090,23 +3090,23 @@
       <c r="E29" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="F29" s="2" t="s">
+      <c r="F29" t="s">
+        <v>35</v>
+      </c>
+      <c r="G29" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="G29" s="2" t="s">
+      <c r="H29" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="J29" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="H29" t="s">
-        <v>35</v>
-      </c>
-      <c r="I29" s="2" t="s">
+      <c r="K29" s="2" t="s">
         <v>379</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="K29" s="2" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3125,23 +3125,23 @@
       <c r="E30" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="F30" t="s">
+        <v>38</v>
+      </c>
+      <c r="G30" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="H30" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="J30" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="H30" t="s">
-        <v>38</v>
-      </c>
-      <c r="I30" s="2" t="s">
+      <c r="K30" s="2" t="s">
         <v>383</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3160,23 +3160,23 @@
       <c r="E31" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="F31" s="2" t="s">
+      <c r="F31" t="s">
+        <v>39</v>
+      </c>
+      <c r="G31" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="G31" s="2" t="s">
+      <c r="H31" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="J31" s="2" t="s">
         <v>386</v>
       </c>
-      <c r="H31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I31" s="2" t="s">
+      <c r="K31" s="2" t="s">
         <v>387</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>388</v>
-      </c>
-      <c r="K31" s="2" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3195,23 +3195,23 @@
       <c r="E32" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="F32" s="2" t="s">
+      <c r="F32" t="s">
+        <v>40</v>
+      </c>
+      <c r="G32" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="H32" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="J32" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="H32" t="s">
-        <v>40</v>
-      </c>
-      <c r="I32" s="2" t="s">
+      <c r="K32" s="2" t="s">
         <v>391</v>
-      </c>
-      <c r="J32" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="K32" s="2" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3230,23 +3230,23 @@
       <c r="E33" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="F33" t="s">
+        <v>42</v>
+      </c>
+      <c r="G33" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="H33" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="J33" s="2" t="s">
         <v>394</v>
       </c>
-      <c r="H33" t="s">
-        <v>42</v>
-      </c>
-      <c r="I33" s="2" t="s">
+      <c r="K33" s="2" t="s">
         <v>395</v>
-      </c>
-      <c r="J33" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="K33" s="2" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3265,23 +3265,23 @@
       <c r="E34" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="F34" t="s">
+        <v>43</v>
+      </c>
+      <c r="G34" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="H34" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="J34" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="H34" t="s">
-        <v>43</v>
-      </c>
-      <c r="I34" s="2" t="s">
+      <c r="K34" s="2" t="s">
         <v>399</v>
-      </c>
-      <c r="J34" s="2" t="s">
-        <v>400</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3300,23 +3300,23 @@
       <c r="E35" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="F35" t="s">
+        <v>45</v>
+      </c>
+      <c r="G35" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="H35" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="J35" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="H35" t="s">
-        <v>45</v>
-      </c>
-      <c r="I35" s="2" t="s">
+      <c r="K35" s="2" t="s">
         <v>403</v>
-      </c>
-      <c r="J35" s="2" t="s">
-        <v>404</v>
-      </c>
-      <c r="K35" s="2" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3335,23 +3335,23 @@
       <c r="E36" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="F36" s="2" t="s">
+      <c r="F36" t="s">
+        <v>47</v>
+      </c>
+      <c r="G36" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="G36" s="2" t="s">
+      <c r="H36" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="J36" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="H36" t="s">
-        <v>47</v>
-      </c>
-      <c r="I36" s="2" t="s">
+      <c r="K36" s="2" t="s">
         <v>407</v>
-      </c>
-      <c r="J36" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3370,23 +3370,23 @@
       <c r="E37" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="F37" s="2" t="s">
+      <c r="F37" t="s">
+        <v>46</v>
+      </c>
+      <c r="G37" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="G37" s="2" t="s">
+      <c r="H37" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="J37" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="H37" t="s">
-        <v>46</v>
-      </c>
-      <c r="I37" s="2" t="s">
+      <c r="K37" s="2" t="s">
         <v>411</v>
-      </c>
-      <c r="J37" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="K37" s="2" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3405,23 +3405,23 @@
       <c r="E38" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="F38" s="2" t="s">
+      <c r="F38" t="s">
+        <v>49</v>
+      </c>
+      <c r="G38" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="G38" s="2" t="s">
+      <c r="H38" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="J38" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="H38" t="s">
-        <v>49</v>
-      </c>
-      <c r="I38" s="2" t="s">
+      <c r="K38" s="2" t="s">
         <v>415</v>
-      </c>
-      <c r="J38" s="2" t="s">
-        <v>416</v>
-      </c>
-      <c r="K38" s="2" t="s">
-        <v>417</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3440,23 +3440,23 @@
       <c r="E39" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="F39" s="2" t="s">
+      <c r="F39" t="s">
+        <v>50</v>
+      </c>
+      <c r="G39" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="G39" s="2" t="s">
+      <c r="H39" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="J39" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="H39" t="s">
-        <v>50</v>
-      </c>
-      <c r="I39" s="2" t="s">
+      <c r="K39" s="2" t="s">
         <v>419</v>
-      </c>
-      <c r="J39" s="2" t="s">
-        <v>420</v>
-      </c>
-      <c r="K39" s="2" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3475,23 +3475,23 @@
       <c r="E40" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="F40" s="2" t="s">
+      <c r="F40" t="s">
+        <v>51</v>
+      </c>
+      <c r="G40" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="G40" s="2" t="s">
+      <c r="H40" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="J40" s="2" t="s">
         <v>422</v>
       </c>
-      <c r="H40" t="s">
-        <v>51</v>
-      </c>
-      <c r="I40" s="2" t="s">
+      <c r="K40" s="2" t="s">
         <v>423</v>
-      </c>
-      <c r="J40" s="2" t="s">
-        <v>424</v>
-      </c>
-      <c r="K40" s="2" t="s">
-        <v>425</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3510,23 +3510,23 @@
       <c r="E41" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="F41" s="2" t="s">
+      <c r="F41" t="s">
+        <v>52</v>
+      </c>
+      <c r="G41" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="G41" s="2" t="s">
+      <c r="H41" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="J41" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="H41" t="s">
-        <v>52</v>
-      </c>
-      <c r="I41" s="2" t="s">
+      <c r="K41" s="2" t="s">
         <v>427</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>428</v>
-      </c>
-      <c r="K41" s="2" t="s">
-        <v>429</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3545,23 +3545,23 @@
       <c r="E42" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="F42" s="2" t="s">
+      <c r="F42" t="s">
+        <v>54</v>
+      </c>
+      <c r="G42" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="G42" s="2" t="s">
+      <c r="H42" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="J42" s="2" t="s">
         <v>430</v>
       </c>
-      <c r="H42" t="s">
-        <v>54</v>
-      </c>
-      <c r="I42" s="2" t="s">
+      <c r="K42" s="2" t="s">
         <v>431</v>
-      </c>
-      <c r="J42" s="2" t="s">
-        <v>432</v>
-      </c>
-      <c r="K42" s="2" t="s">
-        <v>433</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3580,23 +3580,23 @@
       <c r="E43" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="F43" s="2" t="s">
+      <c r="F43" t="s">
+        <v>55</v>
+      </c>
+      <c r="G43" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="G43" s="2" t="s">
+      <c r="H43" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="J43" s="2" t="s">
         <v>434</v>
       </c>
-      <c r="H43" t="s">
-        <v>55</v>
-      </c>
-      <c r="I43" s="2" t="s">
+      <c r="K43" s="2" t="s">
         <v>435</v>
-      </c>
-      <c r="J43" s="2" t="s">
-        <v>436</v>
-      </c>
-      <c r="K43" s="2" t="s">
-        <v>437</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3615,23 +3615,23 @@
       <c r="E44" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="F44" s="2" t="s">
+      <c r="F44" t="s">
+        <v>57</v>
+      </c>
+      <c r="G44" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="G44" s="2" t="s">
+      <c r="H44" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="J44" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="H44" t="s">
-        <v>57</v>
-      </c>
-      <c r="I44" s="2" t="s">
+      <c r="K44" s="2" t="s">
         <v>439</v>
-      </c>
-      <c r="J44" s="2" t="s">
-        <v>440</v>
-      </c>
-      <c r="K44" s="2" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3650,23 +3650,23 @@
       <c r="E45" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="F45" s="2" t="s">
+      <c r="F45" t="s">
+        <v>58</v>
+      </c>
+      <c r="G45" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="G45" s="2" t="s">
+      <c r="H45" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="J45" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="H45" t="s">
-        <v>58</v>
-      </c>
-      <c r="I45" s="2" t="s">
+      <c r="K45" s="2" t="s">
         <v>443</v>
-      </c>
-      <c r="J45" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="K45" s="2" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3685,23 +3685,23 @@
       <c r="E46" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="F46" s="2" t="s">
+      <c r="F46" t="s">
+        <v>59</v>
+      </c>
+      <c r="G46" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="G46" s="2" t="s">
+      <c r="H46" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="J46" s="2" t="s">
         <v>446</v>
       </c>
-      <c r="H46" t="s">
-        <v>59</v>
-      </c>
-      <c r="I46" s="2" t="s">
+      <c r="K46" s="2" t="s">
         <v>447</v>
-      </c>
-      <c r="J46" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="K46" s="2" t="s">
-        <v>449</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3720,23 +3720,23 @@
       <c r="E47" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="F47" s="2" t="s">
+      <c r="F47" t="s">
+        <v>61</v>
+      </c>
+      <c r="G47" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="G47" s="2" t="s">
+      <c r="H47" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="J47" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="H47" t="s">
-        <v>61</v>
-      </c>
-      <c r="I47" s="2" t="s">
+      <c r="K47" s="2" t="s">
         <v>451</v>
-      </c>
-      <c r="J47" s="2" t="s">
-        <v>452</v>
-      </c>
-      <c r="K47" s="2" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3755,23 +3755,23 @@
       <c r="E48" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="F48" s="2" t="s">
+      <c r="F48" t="s">
+        <v>62</v>
+      </c>
+      <c r="G48" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="G48" s="2" t="s">
+      <c r="H48" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="J48" s="2" t="s">
         <v>454</v>
       </c>
-      <c r="H48" t="s">
-        <v>62</v>
-      </c>
-      <c r="I48" s="2" t="s">
+      <c r="K48" s="2" t="s">
         <v>455</v>
-      </c>
-      <c r="J48" s="2" t="s">
-        <v>456</v>
-      </c>
-      <c r="K48" s="2" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3790,23 +3790,23 @@
       <c r="E49" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="F49" s="2" t="s">
+      <c r="F49" t="s">
+        <v>63</v>
+      </c>
+      <c r="G49" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="G49" s="2" t="s">
+      <c r="H49" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="J49" s="2" t="s">
         <v>458</v>
       </c>
-      <c r="H49" t="s">
-        <v>63</v>
-      </c>
-      <c r="I49" s="2" t="s">
+      <c r="K49" s="2" t="s">
         <v>459</v>
-      </c>
-      <c r="J49" s="2" t="s">
-        <v>460</v>
-      </c>
-      <c r="K49" s="2" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3825,23 +3825,23 @@
       <c r="E50" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="F50" s="2" t="s">
+      <c r="F50" t="s">
+        <v>65</v>
+      </c>
+      <c r="G50" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="G50" s="2" t="s">
+      <c r="H50" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="J50" s="2" t="s">
         <v>462</v>
       </c>
-      <c r="H50" t="s">
-        <v>65</v>
-      </c>
-      <c r="I50" s="2" t="s">
+      <c r="K50" s="2" t="s">
         <v>463</v>
-      </c>
-      <c r="J50" s="2" t="s">
-        <v>464</v>
-      </c>
-      <c r="K50" s="2" t="s">
-        <v>465</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3860,23 +3860,23 @@
       <c r="E51" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="F51" s="2" t="s">
+      <c r="F51" t="s">
+        <v>66</v>
+      </c>
+      <c r="G51" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="G51" s="2" t="s">
+      <c r="H51" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="J51" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="H51" t="s">
-        <v>66</v>
-      </c>
-      <c r="I51" s="2" t="s">
+      <c r="K51" s="2" t="s">
         <v>467</v>
-      </c>
-      <c r="J51" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="K51" s="2" t="s">
-        <v>469</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3895,23 +3895,23 @@
       <c r="E52" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="F52" s="2" t="s">
+      <c r="F52" t="s">
+        <v>67</v>
+      </c>
+      <c r="G52" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="G52" s="2" t="s">
+      <c r="H52" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="J52" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="H52" t="s">
-        <v>67</v>
-      </c>
-      <c r="I52" s="2" t="s">
+      <c r="K52" s="2" t="s">
         <v>471</v>
-      </c>
-      <c r="J52" s="2" t="s">
-        <v>472</v>
-      </c>
-      <c r="K52" s="2" t="s">
-        <v>473</v>
       </c>
     </row>
     <row r="53" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3930,23 +3930,23 @@
       <c r="E53" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="F53" s="2" t="s">
+      <c r="F53" t="s">
+        <v>69</v>
+      </c>
+      <c r="G53" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="G53" s="2" t="s">
+      <c r="H53" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="J53" s="2" t="s">
         <v>474</v>
       </c>
-      <c r="H53" t="s">
-        <v>69</v>
-      </c>
-      <c r="I53" s="2" t="s">
+      <c r="K53" s="2" t="s">
         <v>475</v>
-      </c>
-      <c r="J53" s="2" t="s">
-        <v>476</v>
-      </c>
-      <c r="K53" s="2" t="s">
-        <v>477</v>
       </c>
     </row>
     <row r="54" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3965,23 +3965,23 @@
       <c r="E54" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="F54" s="2" t="s">
+      <c r="F54" t="s">
+        <v>70</v>
+      </c>
+      <c r="G54" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="G54" s="2" t="s">
+      <c r="H54" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="J54" s="2" t="s">
         <v>478</v>
       </c>
-      <c r="H54" t="s">
-        <v>70</v>
-      </c>
-      <c r="I54" s="2" t="s">
+      <c r="K54" s="2" t="s">
         <v>479</v>
-      </c>
-      <c r="J54" s="2" t="s">
-        <v>480</v>
-      </c>
-      <c r="K54" s="2" t="s">
-        <v>481</v>
       </c>
     </row>
     <row r="55" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -4000,23 +4000,23 @@
       <c r="E55" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="F55" s="2" t="s">
+      <c r="F55" t="s">
+        <v>71</v>
+      </c>
+      <c r="G55" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="G55" s="2" t="s">
+      <c r="H55" s="2" t="s">
+        <v>480</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="J55" s="2" t="s">
         <v>482</v>
       </c>
-      <c r="H55" t="s">
-        <v>71</v>
-      </c>
-      <c r="I55" s="2" t="s">
+      <c r="K55" s="2" t="s">
         <v>483</v>
-      </c>
-      <c r="J55" s="2" t="s">
-        <v>484</v>
-      </c>
-      <c r="K55" s="2" t="s">
-        <v>485</v>
       </c>
     </row>
     <row r="56" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -4035,23 +4035,23 @@
       <c r="E56" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="F56" s="2" t="s">
+      <c r="F56" t="s">
+        <v>73</v>
+      </c>
+      <c r="G56" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="G56" s="2" t="s">
+      <c r="H56" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="J56" s="2" t="s">
         <v>486</v>
       </c>
-      <c r="H56" t="s">
-        <v>73</v>
-      </c>
-      <c r="I56" s="2" t="s">
+      <c r="K56" s="2" t="s">
         <v>487</v>
-      </c>
-      <c r="J56" s="2" t="s">
-        <v>488</v>
-      </c>
-      <c r="K56" s="2" t="s">
-        <v>489</v>
       </c>
     </row>
     <row r="57" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -4070,23 +4070,23 @@
       <c r="E57" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="F57" s="2" t="s">
+      <c r="F57" t="s">
+        <v>74</v>
+      </c>
+      <c r="G57" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="G57" s="2" t="s">
+      <c r="H57" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="I57" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="J57" s="2" t="s">
         <v>490</v>
       </c>
-      <c r="H57" t="s">
-        <v>74</v>
-      </c>
-      <c r="I57" s="2" t="s">
+      <c r="K57" s="2" t="s">
         <v>491</v>
-      </c>
-      <c r="J57" s="2" t="s">
-        <v>492</v>
-      </c>
-      <c r="K57" s="2" t="s">
-        <v>493</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -4105,23 +4105,23 @@
       <c r="E58" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="F58" s="2" t="s">
+      <c r="F58" t="s">
+        <v>75</v>
+      </c>
+      <c r="G58" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="G58" s="2" t="s">
+      <c r="H58" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="K58" s="2" t="s">
         <v>494</v>
-      </c>
-      <c r="H58" t="s">
-        <v>75</v>
-      </c>
-      <c r="I58" s="2" t="s">
-        <v>495</v>
-      </c>
-      <c r="J58" s="2" t="s">
-        <v>496</v>
-      </c>
-      <c r="K58" s="2" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -4140,23 +4140,23 @@
       <c r="E59" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="F59" s="2" t="s">
+      <c r="F59" t="s">
+        <v>77</v>
+      </c>
+      <c r="G59" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="G59" s="2" t="s">
+      <c r="H59" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="K59" s="2" t="s">
         <v>498</v>
-      </c>
-      <c r="H59" t="s">
-        <v>77</v>
-      </c>
-      <c r="I59" s="2" t="s">
-        <v>499</v>
-      </c>
-      <c r="J59" s="2" t="s">
-        <v>500</v>
-      </c>
-      <c r="K59" s="2" t="s">
-        <v>501</v>
       </c>
     </row>
     <row r="60" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -4175,23 +4175,23 @@
       <c r="E60" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="F60" s="2" t="s">
+      <c r="F60" t="s">
+        <v>78</v>
+      </c>
+      <c r="G60" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="G60" s="2" t="s">
+      <c r="H60" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="I60" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="K60" s="2" t="s">
         <v>502</v>
-      </c>
-      <c r="H60" t="s">
-        <v>78</v>
-      </c>
-      <c r="I60" s="2" t="s">
-        <v>503</v>
-      </c>
-      <c r="J60" s="2" t="s">
-        <v>504</v>
-      </c>
-      <c r="K60" s="2" t="s">
-        <v>505</v>
       </c>
     </row>
     <row r="61" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -4210,23 +4210,23 @@
       <c r="E61" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="F61" s="2" t="s">
+      <c r="F61" t="s">
+        <v>79</v>
+      </c>
+      <c r="G61" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="G61" s="2" t="s">
+      <c r="H61" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="K61" s="2" t="s">
         <v>506</v>
-      </c>
-      <c r="H61" t="s">
-        <v>79</v>
-      </c>
-      <c r="I61" s="2" t="s">
-        <v>507</v>
-      </c>
-      <c r="J61" s="2" t="s">
-        <v>508</v>
-      </c>
-      <c r="K61" s="2" t="s">
-        <v>509</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -4245,23 +4245,23 @@
       <c r="E62" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="F62" s="2" t="s">
+      <c r="F62" t="s">
+        <v>81</v>
+      </c>
+      <c r="G62" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="G62" s="2" t="s">
+      <c r="H62" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="I62" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="J62" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="K62" s="2" t="s">
         <v>510</v>
-      </c>
-      <c r="H62" t="s">
-        <v>81</v>
-      </c>
-      <c r="I62" s="2" t="s">
-        <v>511</v>
-      </c>
-      <c r="J62" s="2" t="s">
-        <v>512</v>
-      </c>
-      <c r="K62" s="2" t="s">
-        <v>513</v>
       </c>
     </row>
     <row r="63" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -4280,23 +4280,23 @@
       <c r="E63" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="F63" s="2" t="s">
+      <c r="F63" t="s">
+        <v>82</v>
+      </c>
+      <c r="G63" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="G63" s="2" t="s">
+      <c r="H63" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="J63" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="K63" s="2" t="s">
         <v>514</v>
-      </c>
-      <c r="H63" t="s">
-        <v>82</v>
-      </c>
-      <c r="I63" s="2" t="s">
-        <v>515</v>
-      </c>
-      <c r="J63" s="2" t="s">
-        <v>516</v>
-      </c>
-      <c r="K63" s="2" t="s">
-        <v>517</v>
       </c>
     </row>
     <row r="64" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -4315,23 +4315,23 @@
       <c r="E64" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="F64" s="2" t="s">
+      <c r="F64" t="s">
+        <v>83</v>
+      </c>
+      <c r="G64" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="G64" s="2" t="s">
+      <c r="H64" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="J64" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="K64" s="2" t="s">
         <v>518</v>
-      </c>
-      <c r="H64" t="s">
-        <v>83</v>
-      </c>
-      <c r="I64" s="2" t="s">
-        <v>519</v>
-      </c>
-      <c r="J64" s="2" t="s">
-        <v>520</v>
-      </c>
-      <c r="K64" s="2" t="s">
-        <v>521</v>
       </c>
     </row>
     <row r="65" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -4350,23 +4350,23 @@
       <c r="E65" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="F65" s="2" t="s">
+      <c r="F65" t="s">
+        <v>84</v>
+      </c>
+      <c r="G65" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="G65" s="2" t="s">
+      <c r="H65" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="J65" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="K65" s="2" t="s">
         <v>522</v>
-      </c>
-      <c r="H65" t="s">
-        <v>84</v>
-      </c>
-      <c r="I65" s="2" t="s">
-        <v>523</v>
-      </c>
-      <c r="J65" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="K65" s="2" t="s">
-        <v>525</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v2.5 Rebranding to YAY
</commit_message>
<xml_diff>
--- a/.audio_ban_1.1.xlsx
+++ b/.audio_ban_1.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\nbs\yay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB2425D3-B406-4623-B4DF-EDEC7A72CAC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01CA9423-CD1B-49CB-A5B7-DE7C1997171B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3380" yWindow="3380" windowWidth="19200" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="546">
   <si>
     <t>Trigger / Filename Prefix</t>
   </si>
@@ -1725,6 +1725,24 @@
   </si>
   <si>
     <t>You ain't catchin' me now!</t>
+  </si>
+  <si>
+    <t>Designation</t>
+  </si>
+  <si>
+    <t>ac</t>
+  </si>
+  <si>
+    <t>jv</t>
+  </si>
+  <si>
+    <t>pf</t>
+  </si>
+  <si>
+    <t>cb</t>
+  </si>
+  <si>
+    <t>df</t>
   </si>
 </sst>
 </file>
@@ -1805,7 +1823,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
@@ -1820,6 +1838,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -2102,12 +2123,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="33.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2127,114 +2148,108 @@
         <v>86</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:11" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="K1" s="1" t="s">
+      <c r="G2" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="182.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="s">
+      <c r="K2" s="6"/>
+    </row>
+    <row r="3" spans="1:11" ht="182.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="D2" s="1" t="s">
+      <c r="B3" s="3"/>
+      <c r="D3" s="1" t="s">
         <v>523</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>524</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>525</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>526</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>527</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>528</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>529</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="168.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="1" t="s">
+    <row r="4" spans="1:11" ht="168.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="D3" s="2" t="s">
+      <c r="B4" s="3"/>
+      <c r="D4" s="2" t="s">
         <v>530</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>531</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>532</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>533</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>534</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>535</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>536</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="140.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="4">
-        <v>100</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:11" ht="140.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
@@ -2242,34 +2257,34 @@
         <v>100</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>2</v>
+        <v>89</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>90</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>93</v>
+        <v>278</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>281</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
@@ -2277,69 +2292,69 @@
         <v>100</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>11</v>
+        <v>92</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>96</v>
+        <v>282</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>285</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="4" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B7" s="4">
         <v>100</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>13</v>
+        <v>95</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>96</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>99</v>
+        <v>286</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>289</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="4" t="s">
         <v>12</v>
       </c>
@@ -2347,34 +2362,34 @@
         <v>100</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>14</v>
+        <v>98</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>99</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>102</v>
+        <v>290</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>293</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
@@ -2382,69 +2397,69 @@
         <v>100</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4">
+        <v>100</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F10" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="K10" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G9" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>299</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="1">
-        <v>25</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>537</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="11" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
         <v>16</v>
       </c>
@@ -2452,34 +2467,34 @@
         <v>25</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>4</v>
+        <v>107</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>108</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>111</v>
+        <v>302</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>305</v>
+        <v>537</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>304</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>16</v>
       </c>
@@ -2487,34 +2502,34 @@
         <v>25</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>5</v>
+        <v>110</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>111</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>114</v>
+        <v>305</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>538</v>
+        <v>307</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>308</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="4" t="s">
         <v>16</v>
       </c>
@@ -2522,34 +2537,34 @@
         <v>25</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>18</v>
+        <v>113</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>114</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>117</v>
+        <v>309</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>312</v>
+        <v>538</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>311</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="4" t="s">
         <v>16</v>
       </c>
@@ -2557,34 +2572,34 @@
         <v>25</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>19</v>
+        <v>116</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>117</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>120</v>
+        <v>312</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>315</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="4" t="s">
         <v>16</v>
       </c>
@@ -2592,34 +2607,34 @@
         <v>25</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>20</v>
+        <v>119</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>120</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>123</v>
+        <v>316</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>319</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="4" t="s">
         <v>16</v>
       </c>
@@ -2627,34 +2642,34 @@
         <v>25</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>21</v>
+        <v>122</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>123</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>126</v>
+        <v>320</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>326</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>323</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="4" t="s">
         <v>16</v>
       </c>
@@ -2662,66 +2677,66 @@
         <v>25</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="1">
+        <v>25</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="F18" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="K18" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>330</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B18" s="1">
-        <v>33</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>332</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>333</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2732,34 +2747,34 @@
         <v>33</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>24</v>
+        <v>131</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>132</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>135</v>
+        <v>332</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>335</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="4" t="s">
         <v>22</v>
       </c>
@@ -2767,69 +2782,69 @@
         <v>33</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>25</v>
+        <v>134</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>135</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>138</v>
+        <v>336</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="K20" s="2" t="s">
-        <v>343</v>
+        <v>339</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B21" s="1">
-        <v>20</v>
-      </c>
-      <c r="C21" t="s">
-        <v>27</v>
+        <v>33</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="F21" t="s">
-        <v>27</v>
+        <v>137</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>138</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>141</v>
+        <v>340</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>346</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>343</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="4" t="s">
         <v>26</v>
       </c>
@@ -2837,31 +2852,31 @@
         <v>20</v>
       </c>
       <c r="C22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="F22" t="s">
-        <v>28</v>
+        <v>140</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>141</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>144</v>
+        <v>344</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="K22" s="2" t="s">
-        <v>351</v>
+        <v>347</v>
+      </c>
+      <c r="K22" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2872,31 +2887,31 @@
         <v>20</v>
       </c>
       <c r="C23" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="F23" t="s">
-        <v>30</v>
+        <v>143</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>147</v>
+        <v>348</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>355</v>
+        <v>351</v>
+      </c>
+      <c r="K23" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2907,34 +2922,34 @@
         <v>20</v>
       </c>
       <c r="C24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="F24" t="s">
-        <v>31</v>
+        <v>146</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>147</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>150</v>
+        <v>352</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>358</v>
-      </c>
-      <c r="K24" s="2" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>355</v>
+      </c>
+      <c r="K24" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="4" t="s">
         <v>26</v>
       </c>
@@ -2942,34 +2957,34 @@
         <v>20</v>
       </c>
       <c r="C25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F25" t="s">
-        <v>32</v>
+        <v>149</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>150</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>153</v>
+        <v>356</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>362</v>
-      </c>
-      <c r="K25" s="2" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>359</v>
+      </c>
+      <c r="K25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="4" t="s">
         <v>26</v>
       </c>
@@ -2977,66 +2992,66 @@
         <v>20</v>
       </c>
       <c r="C26" t="s">
+        <v>32</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="K26" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="1">
+        <v>20</v>
+      </c>
+      <c r="C27" t="s">
         <v>29</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E27" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F27" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="K27" t="s">
         <v>29</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>364</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>365</v>
-      </c>
-      <c r="J26" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B27" s="5">
-        <v>40</v>
-      </c>
-      <c r="C27" t="s">
-        <v>34</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="F27" t="s">
-        <v>34</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>370</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3047,31 +3062,31 @@
         <v>40</v>
       </c>
       <c r="C28" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="F28" t="s">
-        <v>36</v>
+        <v>158</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>159</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>162</v>
+        <v>368</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="K28" s="2" t="s">
-        <v>375</v>
+        <v>371</v>
+      </c>
+      <c r="K28" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3082,69 +3097,69 @@
         <v>40</v>
       </c>
       <c r="C29" t="s">
+        <v>36</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="K29" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B30" s="5">
+        <v>40</v>
+      </c>
+      <c r="C30" t="s">
         <v>35</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="D30" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="E30" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F30" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="K30" t="s">
         <v>35</v>
       </c>
-      <c r="G29" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>376</v>
-      </c>
-      <c r="I29" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="K29" s="2" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B30" s="5">
-        <v>20</v>
-      </c>
-      <c r="C30" t="s">
-        <v>38</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="F30" t="s">
-        <v>38</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="I30" s="2" t="s">
-        <v>381</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>382</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="31" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="4" t="s">
         <v>37</v>
       </c>
@@ -3152,31 +3167,31 @@
         <v>20</v>
       </c>
       <c r="C31" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="F31" t="s">
-        <v>39</v>
+        <v>167</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>168</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>171</v>
+        <v>380</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>386</v>
-      </c>
-      <c r="K31" s="2" t="s">
-        <v>387</v>
+        <v>383</v>
+      </c>
+      <c r="K31" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3187,66 +3202,66 @@
         <v>20</v>
       </c>
       <c r="C32" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="F32" t="s">
-        <v>40</v>
+        <v>170</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>171</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>174</v>
+        <v>384</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="K32" s="2" t="s">
-        <v>391</v>
+        <v>387</v>
+      </c>
+      <c r="K32" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B33" s="5">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="C33" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="F33" t="s">
-        <v>42</v>
+        <v>173</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>174</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>177</v>
+        <v>388</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>394</v>
-      </c>
-      <c r="K33" s="2" t="s">
-        <v>395</v>
+        <v>391</v>
+      </c>
+      <c r="K33" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3257,66 +3272,66 @@
         <v>100</v>
       </c>
       <c r="C34" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="F34" t="s">
-        <v>43</v>
+        <v>176</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>177</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>180</v>
+        <v>392</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>395</v>
+      </c>
+      <c r="K34" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B35" s="5">
         <v>100</v>
       </c>
       <c r="C35" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="F35" t="s">
-        <v>45</v>
+        <v>179</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>180</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>183</v>
+        <v>396</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>402</v>
-      </c>
-      <c r="K35" s="2" t="s">
-        <v>403</v>
+        <v>399</v>
+      </c>
+      <c r="K35" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3327,34 +3342,34 @@
         <v>100</v>
       </c>
       <c r="C36" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="F36" t="s">
-        <v>47</v>
+        <v>182</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>183</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>186</v>
+        <v>400</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>403</v>
+      </c>
+      <c r="K36" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="4" t="s">
         <v>44</v>
       </c>
@@ -3362,104 +3377,104 @@
         <v>100</v>
       </c>
       <c r="C37" t="s">
+        <v>47</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="K37" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A38" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B38" s="5">
+        <v>100</v>
+      </c>
+      <c r="C38" t="s">
         <v>46</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="D38" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="E38" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F38" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="K38" t="s">
         <v>46</v>
       </c>
-      <c r="G37" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="I37" s="2" t="s">
-        <v>409</v>
-      </c>
-      <c r="J37" s="2" t="s">
-        <v>410</v>
-      </c>
-      <c r="K37" s="2" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B38" s="5">
-        <v>75</v>
-      </c>
-      <c r="C38" t="s">
-        <v>49</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="F38" t="s">
-        <v>49</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="I38" s="2" t="s">
-        <v>413</v>
-      </c>
-      <c r="J38" s="2" t="s">
-        <v>414</v>
-      </c>
-      <c r="K38" s="2" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="39" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B39" s="3">
+      <c r="B39" s="5">
         <v>75</v>
       </c>
       <c r="C39" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="F39" t="s">
-        <v>50</v>
+        <v>191</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>192</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>195</v>
+        <v>412</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>418</v>
-      </c>
-      <c r="K39" s="2" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>415</v>
+      </c>
+      <c r="K39" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="4" t="s">
         <v>48</v>
       </c>
@@ -3467,104 +3482,104 @@
         <v>75</v>
       </c>
       <c r="C40" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="F40" t="s">
-        <v>51</v>
+        <v>194</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>195</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>198</v>
+        <v>416</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>422</v>
-      </c>
-      <c r="K40" s="2" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>419</v>
+      </c>
+      <c r="K40" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B41">
+      <c r="B41" s="3">
         <v>75</v>
       </c>
       <c r="C41" t="s">
+        <v>51</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="K41" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A42" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B42">
+        <v>75</v>
+      </c>
+      <c r="C42" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="2" t="s">
+      <c r="D42" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="E41" s="2" t="s">
+      <c r="E42" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="F41" t="s">
+      <c r="F42" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="K42" t="s">
         <v>52</v>
       </c>
-      <c r="G41" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>424</v>
-      </c>
-      <c r="I41" s="2" t="s">
-        <v>425</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>426</v>
-      </c>
-      <c r="K41" s="2" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A42" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B42" s="3">
-        <v>100</v>
-      </c>
-      <c r="C42" t="s">
-        <v>54</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="F42" t="s">
-        <v>54</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="H42" s="2" t="s">
-        <v>428</v>
-      </c>
-      <c r="I42" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="J42" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="K42" s="2" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="43" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A43" s="4" t="s">
         <v>53</v>
       </c>
@@ -3572,69 +3587,69 @@
         <v>100</v>
       </c>
       <c r="C43" t="s">
+        <v>54</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="K43" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A44" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B44" s="3">
+        <v>100</v>
+      </c>
+      <c r="C44" t="s">
         <v>55</v>
       </c>
-      <c r="D43" s="2" t="s">
+      <c r="D44" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="E43" s="2" t="s">
+      <c r="E44" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="F43" t="s">
+      <c r="F44" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="K44" t="s">
         <v>55</v>
       </c>
-      <c r="G43" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="H43" s="2" t="s">
-        <v>432</v>
-      </c>
-      <c r="I43" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="J43" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="K43" s="2" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A44" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B44" s="3">
-        <v>25</v>
-      </c>
-      <c r="C44" t="s">
-        <v>57</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="F44" t="s">
-        <v>57</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="H44" s="2" t="s">
-        <v>436</v>
-      </c>
-      <c r="I44" s="2" t="s">
-        <v>437</v>
-      </c>
-      <c r="J44" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="K44" s="2" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="45" spans="1:11" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A45" s="4" t="s">
         <v>56</v>
       </c>
@@ -3642,101 +3657,101 @@
         <v>25</v>
       </c>
       <c r="C45" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="F45" t="s">
-        <v>58</v>
+        <v>209</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>210</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>213</v>
+        <v>436</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>442</v>
-      </c>
-      <c r="K45" s="2" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>439</v>
+      </c>
+      <c r="K45" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B46">
+      <c r="B46" s="3">
         <v>25</v>
       </c>
       <c r="C46" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="F46" t="s">
-        <v>59</v>
+        <v>212</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>213</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>216</v>
+        <v>440</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>446</v>
-      </c>
-      <c r="K46" s="2" t="s">
-        <v>447</v>
+        <v>443</v>
+      </c>
+      <c r="K46" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B47" s="3">
-        <v>75</v>
+        <v>56</v>
+      </c>
+      <c r="B47">
+        <v>25</v>
       </c>
       <c r="C47" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="F47" t="s">
-        <v>61</v>
+        <v>215</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>216</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>219</v>
+        <v>444</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>450</v>
-      </c>
-      <c r="K47" s="2" t="s">
-        <v>451</v>
+        <v>447</v>
+      </c>
+      <c r="K47" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3747,101 +3762,101 @@
         <v>75</v>
       </c>
       <c r="C48" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="F48" t="s">
-        <v>62</v>
+        <v>218</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>219</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>222</v>
+        <v>448</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>454</v>
-      </c>
-      <c r="K48" s="2" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>451</v>
+      </c>
+      <c r="K48" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B49">
+      <c r="B49" s="3">
         <v>75</v>
       </c>
       <c r="C49" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="F49" t="s">
-        <v>63</v>
+        <v>221</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>222</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>225</v>
+        <v>452</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="K49" s="2" t="s">
-        <v>459</v>
+        <v>455</v>
+      </c>
+      <c r="K49" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A50" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B50" s="3">
+        <v>60</v>
+      </c>
+      <c r="B50">
         <v>75</v>
       </c>
       <c r="C50" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="F50" t="s">
-        <v>65</v>
+        <v>224</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>225</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>228</v>
+        <v>456</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>462</v>
-      </c>
-      <c r="K50" s="2" t="s">
-        <v>463</v>
+        <v>459</v>
+      </c>
+      <c r="K50" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3852,34 +3867,34 @@
         <v>75</v>
       </c>
       <c r="C51" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="F51" t="s">
-        <v>66</v>
+        <v>227</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>228</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>231</v>
+        <v>460</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="K51" s="2" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>463</v>
+      </c>
+      <c r="K51" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A52" s="4" t="s">
         <v>64</v>
       </c>
@@ -3887,69 +3902,69 @@
         <v>75</v>
       </c>
       <c r="C52" t="s">
+        <v>66</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="K52" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A53" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B53" s="3">
+        <v>75</v>
+      </c>
+      <c r="C53" t="s">
         <v>67</v>
       </c>
-      <c r="D52" s="2" t="s">
+      <c r="D53" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="E52" s="2" t="s">
+      <c r="E53" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="F52" t="s">
+      <c r="F53" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="K53" t="s">
         <v>67</v>
       </c>
-      <c r="G52" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="H52" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="I52" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="J52" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="K52" s="2" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A53" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B53" s="3">
-        <v>50</v>
-      </c>
-      <c r="C53" t="s">
-        <v>69</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="F53" t="s">
-        <v>69</v>
-      </c>
-      <c r="G53" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="H53" s="2" t="s">
-        <v>472</v>
-      </c>
-      <c r="I53" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="J53" s="2" t="s">
-        <v>474</v>
-      </c>
-      <c r="K53" s="2" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="54" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A54" s="4" t="s">
         <v>68</v>
       </c>
@@ -3957,34 +3972,34 @@
         <v>50</v>
       </c>
       <c r="C54" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="F54" t="s">
-        <v>70</v>
+        <v>236</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>237</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>240</v>
+        <v>472</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>478</v>
-      </c>
-      <c r="K54" s="2" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>475</v>
+      </c>
+      <c r="K54" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A55" s="4" t="s">
         <v>68</v>
       </c>
@@ -3992,66 +4007,66 @@
         <v>50</v>
       </c>
       <c r="C55" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="F55" t="s">
-        <v>71</v>
+        <v>239</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>240</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>243</v>
+        <v>476</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>482</v>
-      </c>
-      <c r="K55" s="2" t="s">
-        <v>483</v>
+        <v>479</v>
+      </c>
+      <c r="K55" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="56" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="4" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B56" s="3">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C56" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="F56" t="s">
-        <v>73</v>
+        <v>242</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>243</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>246</v>
+        <v>480</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>486</v>
-      </c>
-      <c r="K56" s="2" t="s">
-        <v>487</v>
+        <v>483</v>
+      </c>
+      <c r="K56" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="57" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -4062,31 +4077,31 @@
         <v>25</v>
       </c>
       <c r="C57" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="F57" t="s">
-        <v>74</v>
+        <v>245</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>246</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>249</v>
+        <v>484</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>490</v>
-      </c>
-      <c r="K57" s="2" t="s">
-        <v>491</v>
+        <v>487</v>
+      </c>
+      <c r="K57" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -4097,69 +4112,69 @@
         <v>25</v>
       </c>
       <c r="C58" t="s">
+        <v>74</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="K58" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A59" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B59" s="3">
+        <v>25</v>
+      </c>
+      <c r="C59" t="s">
         <v>75</v>
       </c>
-      <c r="D58" s="2" t="s">
+      <c r="D59" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="E58" s="2" t="s">
+      <c r="E59" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="F58" t="s">
+      <c r="F59" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="K59" t="s">
         <v>75</v>
       </c>
-      <c r="G58" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="H58" s="2" t="s">
-        <v>492</v>
-      </c>
-      <c r="I58" s="2" t="s">
-        <v>539</v>
-      </c>
-      <c r="J58" s="2" t="s">
-        <v>493</v>
-      </c>
-      <c r="K58" s="2" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A59" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B59" s="3">
-        <v>100</v>
-      </c>
-      <c r="C59" t="s">
-        <v>77</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="F59" t="s">
-        <v>77</v>
-      </c>
-      <c r="G59" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="H59" s="2" t="s">
-        <v>495</v>
-      </c>
-      <c r="I59" s="2" t="s">
-        <v>496</v>
-      </c>
-      <c r="J59" s="2" t="s">
-        <v>497</v>
-      </c>
-      <c r="K59" s="2" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="60" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A60" s="4" t="s">
         <v>76</v>
       </c>
@@ -4167,34 +4182,34 @@
         <v>100</v>
       </c>
       <c r="C60" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="F60" t="s">
-        <v>78</v>
+        <v>254</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>255</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>258</v>
+        <v>495</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>501</v>
-      </c>
-      <c r="K60" s="2" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>498</v>
+      </c>
+      <c r="K60" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="4" t="s">
         <v>76</v>
       </c>
@@ -4202,66 +4217,66 @@
         <v>100</v>
       </c>
       <c r="C61" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="F61" t="s">
-        <v>79</v>
+        <v>257</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>258</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>261</v>
+        <v>499</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>505</v>
-      </c>
-      <c r="K61" s="2" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>502</v>
+      </c>
+      <c r="K61" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A62" s="4" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B62" s="3">
         <v>100</v>
       </c>
       <c r="C62" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="F62" t="s">
-        <v>81</v>
+        <v>260</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>261</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>264</v>
+        <v>503</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="J62" s="2" t="s">
-        <v>509</v>
-      </c>
-      <c r="K62" s="2" t="s">
-        <v>510</v>
+        <v>506</v>
+      </c>
+      <c r="K62" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="63" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -4272,34 +4287,34 @@
         <v>100</v>
       </c>
       <c r="C63" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="F63" t="s">
-        <v>82</v>
+        <v>263</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>264</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>267</v>
+        <v>507</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="I63" s="2" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="J63" s="2" t="s">
-        <v>513</v>
-      </c>
-      <c r="K63" s="2" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>510</v>
+      </c>
+      <c r="K63" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" ht="98.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A64" s="4" t="s">
         <v>80</v>
       </c>
@@ -4307,31 +4322,31 @@
         <v>100</v>
       </c>
       <c r="C64" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="F64" t="s">
-        <v>83</v>
+        <v>266</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>267</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>270</v>
+        <v>511</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="I64" s="2" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="J64" s="2" t="s">
-        <v>517</v>
-      </c>
-      <c r="K64" s="2" t="s">
-        <v>518</v>
+        <v>514</v>
+      </c>
+      <c r="K64" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="65" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -4342,31 +4357,66 @@
         <v>100</v>
       </c>
       <c r="C65" t="s">
+        <v>83</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="J65" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="K65" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="112.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A66" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B66" s="3">
+        <v>100</v>
+      </c>
+      <c r="C66" t="s">
         <v>84</v>
       </c>
-      <c r="D65" s="2" t="s">
+      <c r="D66" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="E65" s="2" t="s">
+      <c r="E66" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="F65" t="s">
+      <c r="F66" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="I66" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="J66" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="K66" t="s">
         <v>84</v>
-      </c>
-      <c r="G65" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="H65" s="2" t="s">
-        <v>519</v>
-      </c>
-      <c r="I65" s="2" t="s">
-        <v>520</v>
-      </c>
-      <c r="J65" s="2" t="s">
-        <v>521</v>
-      </c>
-      <c r="K65" s="2" t="s">
-        <v>522</v>
       </c>
     </row>
   </sheetData>

</xml_diff>